<commit_message>
GreenHub Alpha 0.2 Checkpoint 1
</commit_message>
<xml_diff>
--- a/Greenhub/results/integrated_greenhub_report.xlsx
+++ b/Greenhub/results/integrated_greenhub_report.xlsx
@@ -522,7 +522,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29T11:34:23.896403+00:00</t>
+          <t>2026-07-29T16:49:41.688327+00:00</t>
         </is>
       </c>
     </row>
@@ -534,7 +534,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>6ba0493c007df20c9f94dbf78b9214911c738044</t>
+          <t>39dcf17581a253e3b2d8e2a68a4f759fb68a832e</t>
         </is>
       </c>
     </row>
@@ -3815,7 +3815,7 @@
         </is>
       </c>
       <c r="C8" s="8" t="n">
-        <v>243.6194401251267</v>
+        <v>243.6194401251268</v>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
@@ -4674,7 +4674,7 @@
         </is>
       </c>
       <c r="C24" s="8" t="n">
-        <v>0.5824700352607181</v>
+        <v>0.5824700352607179</v>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
@@ -4699,7 +4699,7 @@
         </is>
       </c>
       <c r="C25" s="9" t="n">
-        <v>0.5824700352607181</v>
+        <v>0.5824700352607179</v>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
@@ -5367,7 +5367,7 @@
         </is>
       </c>
       <c r="C15" s="9" t="n">
-        <v>243.6194401251267</v>
+        <v>243.6194401251268</v>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
@@ -5392,7 +5392,7 @@
         </is>
       </c>
       <c r="C16" s="8" t="n">
-        <v>243.6194401251267</v>
+        <v>243.6194401251268</v>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
@@ -5417,7 +5417,7 @@
         </is>
       </c>
       <c r="C17" s="9" t="n">
-        <v>3.20719178564155</v>
+        <v>3.207191785641549</v>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
@@ -6229,7 +6229,7 @@
         </is>
       </c>
       <c r="B2" s="4" t="n">
-        <v>403.9938456027056</v>
+        <v>403.9938456027057</v>
       </c>
       <c r="C2" s="4" t="n">
         <v>403.993845606615</v>
@@ -6251,8 +6251,8 @@
       </c>
       <c r="B3" s="3" t="inlineStr"/>
       <c r="C3" s="3" t="inlineStr"/>
-      <c r="D3" s="5" t="n">
-        <v>-2.842170943040401e-14</v>
+      <c r="D3" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
@@ -6272,8 +6272,8 @@
       <c r="C4" s="4" t="n">
         <v>1.386375062620755</v>
       </c>
-      <c r="D4" s="4" t="n">
-        <v>-2.220446049250313e-16</v>
+      <c r="D4" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
@@ -6288,13 +6288,13 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>27.55412883179702</v>
+        <v>27.55412883179703</v>
       </c>
       <c r="C5" s="5" t="n">
-        <v>27.55412883179702</v>
-      </c>
-      <c r="D5" s="5" t="n">
-        <v>-3.552713678800501e-15</v>
+        <v>27.55412883179703</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
@@ -6354,10 +6354,10 @@
         <v>0.07783134269112162</v>
       </c>
       <c r="C8" s="4" t="n">
-        <v>0.07783134269112163</v>
-      </c>
-      <c r="D8" s="4" t="n">
-        <v>-1.387778780781446e-17</v>
+        <v>0.07783134269112162</v>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
@@ -6419,8 +6419,8 @@
       <c r="C11" s="5" t="n">
         <v>0.3211609710309256</v>
       </c>
-      <c r="D11" s="5" t="n">
-        <v>-5.551115123125783e-17</v>
+      <c r="D11" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
@@ -6613,13 +6613,13 @@
         </is>
       </c>
       <c r="C3" s="5" t="n">
-        <v>0.5824700352607181</v>
+        <v>0.5824700352607179</v>
       </c>
       <c r="D3" s="5" t="n">
         <v>6.616303420863869e-05</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>0.5824038722265095</v>
+        <v>0.5824038722265094</v>
       </c>
       <c r="F3" s="5" t="n">
         <v>288.15</v>
@@ -6687,13 +6687,13 @@
         </is>
       </c>
       <c r="C5" s="5" t="n">
-        <v>243.6194401251267</v>
+        <v>243.6194401251268</v>
       </c>
       <c r="D5" s="5" t="n">
         <v>239.2768287044296</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>4.342611420697182</v>
+        <v>4.342611420697153</v>
       </c>
       <c r="F5" s="5" t="n">
         <v>308.15</v>
@@ -6724,10 +6724,10 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>3.20719178564155</v>
+        <v>3.207191785641549</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>2.56575342851324</v>
+        <v>2.565753428513239</v>
       </c>
       <c r="E6" s="4" t="n">
         <v>0.64143835712831</v>
@@ -6838,7 +6838,7 @@
         <v>238.9215814627983</v>
       </c>
       <c r="D9" s="5" t="n">
-        <v>235.6550167638068</v>
+        <v>235.6550167638069</v>
       </c>
       <c r="E9" s="5" t="n">
         <v>3.266564698991488</v>
@@ -7662,7 +7662,7 @@
         </is>
       </c>
       <c r="C28" s="4" t="n">
-        <v>0.1920746276850114</v>
+        <v>0.1920746276850118</v>
       </c>
       <c r="D28" s="2" t="n">
         <v>0</v>
@@ -7695,7 +7695,7 @@
         <v>0</v>
       </c>
       <c r="F29" s="5" t="n">
-        <v>0.1536597021480091</v>
+        <v>0.1536597021480096</v>
       </c>
     </row>
     <row r="30">
@@ -7998,7 +7998,7 @@
         </is>
       </c>
       <c r="C42" s="4" t="n">
-        <v>0.01202301653950286</v>
+        <v>0.01202301653950287</v>
       </c>
       <c r="D42" s="2" t="n">
         <v>0</v>
@@ -8124,7 +8124,7 @@
         <v>0</v>
       </c>
       <c r="E47" s="5" t="n">
-        <v>7.036149712795237</v>
+        <v>7.036149712795238</v>
       </c>
       <c r="F47" s="3" t="n">
         <v>0</v>

</xml_diff>